<commit_message>
tuesday run for week 7
</commit_message>
<xml_diff>
--- a/bet_tracker.xlsx
+++ b/bet_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\OneDrive - Hunter - CUNY\Documents\Football-DNA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFF46E05-2522-4543-8CD1-9CB3322D68CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D030F4CE-F8C4-4332-991F-9FF57374BC7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{036D8D07-6DDF-4B12-BC99-5F86D347E4BA}"/>
   </bookViews>
@@ -1364,6 +1364,9 @@
       <c r="F33">
         <v>8</v>
       </c>
+      <c r="G33">
+        <v>15.84</v>
+      </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34">
@@ -1406,6 +1409,9 @@
       </c>
       <c r="F35">
         <v>11</v>
+      </c>
+      <c r="G35">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
initial week 7 run
</commit_message>
<xml_diff>
--- a/bet_tracker.xlsx
+++ b/bet_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\OneDrive - Hunter - CUNY\Documents\Football-DNA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D030F4CE-F8C4-4332-991F-9FF57374BC7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A864D06-326D-44AA-9417-1478ACD277C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{036D8D07-6DDF-4B12-BC99-5F86D347E4BA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="74">
   <si>
     <t>week</t>
   </si>
@@ -231,6 +231,36 @@
   </si>
   <si>
     <t>ARI_LA</t>
+  </si>
+  <si>
+    <t>PIT_NO</t>
+  </si>
+  <si>
+    <t>O43.5</t>
+  </si>
+  <si>
+    <t>MIA_NYJ</t>
+  </si>
+  <si>
+    <t>NYJ -4.5</t>
+  </si>
+  <si>
+    <t>DEN_ARI</t>
+  </si>
+  <si>
+    <t>ARI +4.5</t>
+  </si>
+  <si>
+    <t>LA_LV</t>
+  </si>
+  <si>
+    <t>LV +5.5</t>
+  </si>
+  <si>
+    <t>KC_SEA</t>
+  </si>
+  <si>
+    <t>KC +2.5</t>
   </si>
 </sst>
 </file>
@@ -603,7 +633,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD4680C9-A68E-48F0-BAC6-3E37E0DEC4C2}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="10.08984375" bestFit="1" customWidth="1"/>
@@ -1414,6 +1444,167 @@
         <v>0</v>
       </c>
     </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>7</v>
+      </c>
+      <c r="B36" s="1">
+        <v>46314</v>
+      </c>
+      <c r="C36" t="s">
+        <v>64</v>
+      </c>
+      <c r="D36" t="s">
+        <v>65</v>
+      </c>
+      <c r="E36">
+        <v>-118</v>
+      </c>
+      <c r="F36">
+        <v>10</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>7</v>
+      </c>
+      <c r="B37" s="1">
+        <v>46314</v>
+      </c>
+      <c r="C37" t="s">
+        <v>66</v>
+      </c>
+      <c r="D37" t="s">
+        <v>67</v>
+      </c>
+      <c r="E37">
+        <v>-112</v>
+      </c>
+      <c r="F37">
+        <v>11</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>7</v>
+      </c>
+      <c r="B38" s="1">
+        <v>46314</v>
+      </c>
+      <c r="C38" t="s">
+        <v>68</v>
+      </c>
+      <c r="D38" t="s">
+        <v>65</v>
+      </c>
+      <c r="E38">
+        <v>-102</v>
+      </c>
+      <c r="F38">
+        <v>8</v>
+      </c>
+      <c r="G38">
+        <v>15.84</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>7</v>
+      </c>
+      <c r="B39" s="1">
+        <v>46314</v>
+      </c>
+      <c r="C39" t="s">
+        <v>68</v>
+      </c>
+      <c r="D39" t="s">
+        <v>69</v>
+      </c>
+      <c r="E39">
+        <v>-115</v>
+      </c>
+      <c r="F39">
+        <v>14</v>
+      </c>
+      <c r="G39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>7</v>
+      </c>
+      <c r="B40" s="1">
+        <v>46314</v>
+      </c>
+      <c r="C40" t="s">
+        <v>70</v>
+      </c>
+      <c r="D40" t="s">
+        <v>71</v>
+      </c>
+      <c r="E40">
+        <v>-110</v>
+      </c>
+      <c r="F40">
+        <v>18</v>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>7</v>
+      </c>
+      <c r="B41" s="1">
+        <v>46314</v>
+      </c>
+      <c r="C41" t="s">
+        <v>72</v>
+      </c>
+      <c r="D41" t="s">
+        <v>6</v>
+      </c>
+      <c r="E41">
+        <v>-105</v>
+      </c>
+      <c r="F41">
+        <v>9</v>
+      </c>
+      <c r="G41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>7</v>
+      </c>
+      <c r="B42" s="1">
+        <v>46314</v>
+      </c>
+      <c r="C42" t="s">
+        <v>72</v>
+      </c>
+      <c r="D42" t="s">
+        <v>73</v>
+      </c>
+      <c r="E42">
+        <v>-115</v>
+      </c>
+      <c r="F42">
+        <v>5</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>